<commit_message>
Filled blank document reference cells
Blank "Standards Document Reference" cells filled (rows 24-35)
</commit_message>
<xml_diff>
--- a/Documents/S-158-98/2.0.0/WD-158_98_2_0_0_20260831.xlsx
+++ b/Documents/S-158-98/2.0.0/WD-158_98_2_0_0_20260831.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\work\git\S-100-Validation-Checks\Documents\S-158-98\2.0.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14889900-32AD-4A98-B75C-195D99675A12}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{352AD4A6-8738-40CC-961F-AE2FCBEAE731}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="28110" windowHeight="18240" activeTab="1" xr2:uid="{D500D42E-56ED-44C2-B321-3F3845968AA3}"/>
   </bookViews>
@@ -175,7 +175,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="324">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="512" uniqueCount="324">
   <si>
     <t>Classification</t>
   </si>
@@ -2119,18 +2119,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2191,6 +2179,18 @@
     <xf numFmtId="0" fontId="23" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -2577,14 +2577,14 @@
   <sheetData>
     <row r="1" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:8" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="95" t="s">
+      <c r="B2" s="118" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="96"/>
-      <c r="D2" s="96"/>
-      <c r="E2" s="96"/>
-      <c r="F2" s="96"/>
-      <c r="G2" s="97"/>
+      <c r="C2" s="119"/>
+      <c r="D2" s="119"/>
+      <c r="E2" s="119"/>
+      <c r="F2" s="119"/>
+      <c r="G2" s="120"/>
       <c r="H2" s="7"/>
     </row>
     <row r="3" spans="2:8" s="6" customFormat="1" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
@@ -2710,7 +2710,7 @@
       <c r="G12" s="9"/>
     </row>
     <row r="13" spans="2:8" s="6" customFormat="1" ht="31.5" x14ac:dyDescent="0.25">
-      <c r="B13" s="94" t="s">
+      <c r="B13" s="117" t="s">
         <v>14</v>
       </c>
       <c r="C13" s="57" t="s">
@@ -2724,7 +2724,7 @@
       <c r="G13" s="9"/>
     </row>
     <row r="14" spans="2:8" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B14" s="94"/>
+      <c r="B14" s="117"/>
       <c r="C14" s="60" t="s">
         <v>68</v>
       </c>
@@ -2736,7 +2736,7 @@
       <c r="G14" s="9"/>
     </row>
     <row r="15" spans="2:8" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B15" s="94"/>
+      <c r="B15" s="117"/>
       <c r="C15" s="58" t="s">
         <v>35</v>
       </c>
@@ -2748,7 +2748,7 @@
       <c r="G15" s="9"/>
     </row>
     <row r="16" spans="2:8" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B16" s="94"/>
+      <c r="B16" s="117"/>
       <c r="C16" s="59" t="s">
         <v>36</v>
       </c>
@@ -2760,7 +2760,7 @@
       <c r="G16" s="9"/>
     </row>
     <row r="17" spans="2:7" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B17" s="94"/>
+      <c r="B17" s="117"/>
       <c r="C17" s="60" t="s">
         <v>37</v>
       </c>
@@ -2772,7 +2772,7 @@
       <c r="G17" s="9"/>
     </row>
     <row r="18" spans="2:7" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B18" s="94"/>
+      <c r="B18" s="117"/>
       <c r="C18" s="74" t="s">
         <v>69</v>
       </c>
@@ -2784,7 +2784,7 @@
       <c r="G18" s="9"/>
     </row>
     <row r="19" spans="2:7" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B19" s="94"/>
+      <c r="B19" s="117"/>
       <c r="C19" s="73" t="s">
         <v>70</v>
       </c>
@@ -2796,7 +2796,7 @@
       <c r="G19" s="9"/>
     </row>
     <row r="20" spans="2:7" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B20" s="94"/>
+      <c r="B20" s="117"/>
       <c r="C20" s="73" t="s">
         <v>167</v>
       </c>
@@ -2808,7 +2808,7 @@
       <c r="G20" s="9"/>
     </row>
     <row r="21" spans="2:7" s="6" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="B21" s="94"/>
+      <c r="B21" s="117"/>
       <c r="C21" s="65" t="s">
         <v>168</v>
       </c>
@@ -2820,7 +2820,7 @@
       <c r="G21" s="9"/>
     </row>
     <row r="22" spans="2:7" s="6" customFormat="1" ht="20.45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="94"/>
+      <c r="B22" s="117"/>
       <c r="C22" s="66"/>
       <c r="D22" s="68"/>
       <c r="E22" s="68"/>
@@ -2873,62 +2873,62 @@
     <col min="12" max="12" width="21" style="33" customWidth="1"/>
     <col min="13" max="13" width="21.7109375" style="33" customWidth="1"/>
     <col min="14" max="14" width="12.5703125" style="2" customWidth="1"/>
-    <col min="15" max="15" width="25.5703125" style="108" customWidth="1"/>
+    <col min="15" max="15" width="25.5703125" style="104" customWidth="1"/>
     <col min="16" max="16" width="16.28515625" style="2" customWidth="1"/>
     <col min="17" max="17" width="33.28515625" style="2" customWidth="1"/>
     <col min="18" max="16384" width="8.7109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="106" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A1" s="101" t="s">
+    <row r="1" spans="1:17" s="102" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A1" s="97" t="s">
         <v>11</v>
       </c>
-      <c r="B1" s="101" t="s">
+      <c r="B1" s="97" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="101" t="s">
+      <c r="C1" s="97" t="s">
         <v>0</v>
       </c>
-      <c r="D1" s="101" t="s">
+      <c r="D1" s="97" t="s">
         <v>10</v>
       </c>
-      <c r="E1" s="101" t="s">
+      <c r="E1" s="97" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="101" t="s">
+      <c r="F1" s="97" t="s">
         <v>7</v>
       </c>
-      <c r="G1" s="101" t="s">
+      <c r="G1" s="97" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="102" t="s">
+      <c r="H1" s="98" t="s">
         <v>8</v>
       </c>
-      <c r="I1" s="103" t="s">
+      <c r="I1" s="99" t="s">
         <v>2</v>
       </c>
-      <c r="J1" s="103" t="s">
+      <c r="J1" s="99" t="s">
         <v>3</v>
       </c>
-      <c r="K1" s="103" t="s">
+      <c r="K1" s="99" t="s">
         <v>5</v>
       </c>
-      <c r="L1" s="104" t="s">
+      <c r="L1" s="100" t="s">
         <v>33</v>
       </c>
-      <c r="M1" s="104" t="s">
+      <c r="M1" s="100" t="s">
         <v>62</v>
       </c>
-      <c r="N1" s="105" t="s">
+      <c r="N1" s="101" t="s">
         <v>83</v>
       </c>
-      <c r="O1" s="107" t="s">
+      <c r="O1" s="103" t="s">
         <v>196</v>
       </c>
-      <c r="P1" s="99" t="s">
+      <c r="P1" s="95" t="s">
         <v>197</v>
       </c>
-      <c r="Q1" s="100" t="s">
+      <c r="Q1" s="96" t="s">
         <v>198</v>
       </c>
     </row>
@@ -2951,16 +2951,16 @@
       <c r="F2" s="30" t="s">
         <v>173</v>
       </c>
-      <c r="G2" s="98" t="s">
+      <c r="G2" s="94" t="s">
         <v>199</v>
       </c>
-      <c r="H2" s="109" t="s">
+      <c r="H2" s="105" t="s">
         <v>200</v>
       </c>
-      <c r="I2" s="98" t="s">
+      <c r="I2" s="94" t="s">
         <v>71</v>
       </c>
-      <c r="J2" s="110" t="s">
+      <c r="J2" s="106" t="s">
         <v>72</v>
       </c>
       <c r="K2" s="80"/>
@@ -3003,8 +3003,8 @@
       <c r="I3" s="41" t="s">
         <v>128</v>
       </c>
-      <c r="J3" s="110"/>
-      <c r="K3" s="110" t="s">
+      <c r="J3" s="106"/>
+      <c r="K3" s="106" t="s">
         <v>72</v>
       </c>
       <c r="L3" s="33" t="s">
@@ -3016,7 +3016,7 @@
       <c r="N3" s="84" t="s">
         <v>95</v>
       </c>
-      <c r="O3" s="108" t="s">
+      <c r="O3" s="104" t="s">
         <v>203</v>
       </c>
       <c r="Q3" s="2" t="s">
@@ -3030,7 +3030,7 @@
       <c r="B4" s="33" t="s">
         <v>148</v>
       </c>
-      <c r="C4" s="111" t="s">
+      <c r="C4" s="107" t="s">
         <v>112</v>
       </c>
       <c r="D4" s="32" t="s">
@@ -3048,10 +3048,10 @@
       <c r="H4" s="56" t="s">
         <v>205</v>
       </c>
-      <c r="I4" s="98" t="s">
+      <c r="I4" s="94" t="s">
         <v>71</v>
       </c>
-      <c r="J4" s="110" t="s">
+      <c r="J4" s="106" t="s">
         <v>72</v>
       </c>
       <c r="K4" s="80"/>
@@ -3064,10 +3064,10 @@
       <c r="N4" s="84" t="s">
         <v>95</v>
       </c>
-      <c r="O4" s="108" t="s">
+      <c r="O4" s="104" t="s">
         <v>204</v>
       </c>
-      <c r="Q4" s="108" t="s">
+      <c r="Q4" s="104" t="s">
         <v>207</v>
       </c>
     </row>
@@ -3078,7 +3078,7 @@
       <c r="B5" s="33" t="s">
         <v>149</v>
       </c>
-      <c r="C5" s="111" t="s">
+      <c r="C5" s="107" t="s">
         <v>112</v>
       </c>
       <c r="D5" s="32" t="s">
@@ -3096,10 +3096,10 @@
       <c r="H5" s="56" t="s">
         <v>209</v>
       </c>
-      <c r="I5" s="98" t="s">
+      <c r="I5" s="94" t="s">
         <v>71</v>
       </c>
-      <c r="J5" s="110" t="s">
+      <c r="J5" s="106" t="s">
         <v>72</v>
       </c>
       <c r="K5" s="80"/>
@@ -3112,7 +3112,7 @@
       <c r="N5" s="84" t="s">
         <v>95</v>
       </c>
-      <c r="Q5" s="108" t="s">
+      <c r="Q5" s="104" t="s">
         <v>212</v>
       </c>
     </row>
@@ -3123,7 +3123,7 @@
       <c r="B6" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="C6" s="111" t="s">
+      <c r="C6" s="107" t="s">
         <v>112</v>
       </c>
       <c r="D6" s="32" t="s">
@@ -3138,13 +3138,13 @@
       <c r="G6" s="41" t="s">
         <v>101</v>
       </c>
-      <c r="H6" s="109" t="s">
+      <c r="H6" s="105" t="s">
         <v>210</v>
       </c>
-      <c r="I6" s="98" t="s">
+      <c r="I6" s="94" t="s">
         <v>71</v>
       </c>
-      <c r="J6" s="110" t="s">
+      <c r="J6" s="106" t="s">
         <v>72</v>
       </c>
       <c r="K6" s="80"/>
@@ -3157,7 +3157,7 @@
       <c r="N6" s="84" t="s">
         <v>95</v>
       </c>
-      <c r="Q6" s="108" t="s">
+      <c r="Q6" s="104" t="s">
         <v>212</v>
       </c>
     </row>
@@ -3183,13 +3183,13 @@
       <c r="G7" s="41" t="s">
         <v>101</v>
       </c>
-      <c r="H7" s="109" t="s">
+      <c r="H7" s="105" t="s">
         <v>213</v>
       </c>
-      <c r="I7" s="98" t="s">
+      <c r="I7" s="94" t="s">
         <v>71</v>
       </c>
-      <c r="J7" s="110" t="s">
+      <c r="J7" s="106" t="s">
         <v>72</v>
       </c>
       <c r="K7" s="80"/>
@@ -3200,7 +3200,7 @@
         <v>63</v>
       </c>
       <c r="N7" s="84"/>
-      <c r="Q7" s="108"/>
+      <c r="Q7" s="104"/>
     </row>
     <row r="8" spans="1:17" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="40" t="s">
@@ -3225,7 +3225,7 @@
         <v>171</v>
       </c>
       <c r="H8" s="89"/>
-      <c r="I8" s="98" t="s">
+      <c r="I8" s="94" t="s">
         <v>71</v>
       </c>
       <c r="J8" s="90"/>
@@ -3268,11 +3268,11 @@
       <c r="H9" s="89" t="s">
         <v>134</v>
       </c>
-      <c r="I9" s="98" t="s">
+      <c r="I9" s="94" t="s">
         <v>71</v>
       </c>
       <c r="J9" s="92"/>
-      <c r="K9" s="112" t="s">
+      <c r="K9" s="108" t="s">
         <v>72</v>
       </c>
       <c r="L9" s="88" t="s">
@@ -3308,13 +3308,13 @@
       <c r="G10" s="41" t="s">
         <v>101</v>
       </c>
-      <c r="H10" s="109" t="s">
+      <c r="H10" s="105" t="s">
         <v>215</v>
       </c>
-      <c r="I10" s="98" t="s">
+      <c r="I10" s="94" t="s">
         <v>71</v>
       </c>
-      <c r="J10" s="112" t="s">
+      <c r="J10" s="108" t="s">
         <v>72</v>
       </c>
       <c r="K10" s="92"/>
@@ -3347,10 +3347,10 @@
       <c r="H11" s="89" t="s">
         <v>216</v>
       </c>
-      <c r="I11" s="98" t="s">
+      <c r="I11" s="94" t="s">
         <v>71</v>
       </c>
-      <c r="J11" s="112" t="s">
+      <c r="J11" s="108" t="s">
         <v>72</v>
       </c>
       <c r="K11" s="92"/>
@@ -3387,10 +3387,10 @@
       <c r="H12" s="89" t="s">
         <v>216</v>
       </c>
-      <c r="I12" s="98" t="s">
+      <c r="I12" s="94" t="s">
         <v>71</v>
       </c>
-      <c r="J12" s="112" t="s">
+      <c r="J12" s="108" t="s">
         <v>72</v>
       </c>
       <c r="K12" s="92"/>
@@ -3424,13 +3424,13 @@
       <c r="G13" s="41" t="s">
         <v>217</v>
       </c>
-      <c r="H13" s="109" t="s">
+      <c r="H13" s="105" t="s">
         <v>218</v>
       </c>
-      <c r="I13" s="98" t="s">
+      <c r="I13" s="94" t="s">
         <v>71</v>
       </c>
-      <c r="J13" s="112" t="s">
+      <c r="J13" s="108" t="s">
         <v>72</v>
       </c>
       <c r="K13" s="92"/>
@@ -3464,13 +3464,13 @@
       <c r="G14" s="41" t="s">
         <v>217</v>
       </c>
-      <c r="H14" s="109" t="s">
+      <c r="H14" s="105" t="s">
         <v>218</v>
       </c>
-      <c r="I14" s="98" t="s">
+      <c r="I14" s="94" t="s">
         <v>71</v>
       </c>
-      <c r="J14" s="112" t="s">
+      <c r="J14" s="108" t="s">
         <v>72</v>
       </c>
       <c r="K14" s="92"/>
@@ -3510,7 +3510,7 @@
       <c r="I15" s="50" t="s">
         <v>128</v>
       </c>
-      <c r="J15" s="112"/>
+      <c r="J15" s="108"/>
       <c r="K15" s="92"/>
       <c r="L15" s="88" t="s">
         <v>41</v>
@@ -3683,619 +3683,645 @@
         <v>220</v>
       </c>
     </row>
-    <row r="20" spans="1:17" s="118" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A20" s="98" t="s">
+    <row r="20" spans="1:17" s="114" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A20" s="94" t="s">
         <v>291</v>
       </c>
-      <c r="B20" s="113" t="s">
+      <c r="B20" s="109" t="s">
         <v>292</v>
       </c>
-      <c r="C20" s="111" t="s">
+      <c r="C20" s="107" t="s">
         <v>114</v>
       </c>
-      <c r="D20" s="114" t="s">
+      <c r="D20" s="110" t="s">
         <v>46</v>
       </c>
-      <c r="E20" s="115" t="s">
+      <c r="E20" s="111" t="s">
         <v>294</v>
       </c>
-      <c r="F20" s="98" t="s">
+      <c r="F20" s="94" t="s">
         <v>65</v>
       </c>
-      <c r="G20" s="98" t="s">
+      <c r="G20" s="94" t="s">
         <v>227</v>
       </c>
-      <c r="H20" s="109" t="s">
+      <c r="H20" s="105" t="s">
         <v>293</v>
       </c>
-      <c r="I20" s="98" t="s">
+      <c r="I20" s="94" t="s">
         <v>72</v>
       </c>
-      <c r="J20" s="110"/>
-      <c r="K20" s="110"/>
-      <c r="L20" s="113" t="s">
+      <c r="J20" s="106"/>
+      <c r="K20" s="106"/>
+      <c r="L20" s="109" t="s">
         <v>39</v>
       </c>
-      <c r="M20" s="116" t="s">
+      <c r="M20" s="112" t="s">
         <v>275</v>
       </c>
-      <c r="N20" s="117"/>
-      <c r="O20" s="108"/>
-      <c r="P20" s="108"/>
-      <c r="Q20" s="108"/>
-    </row>
-    <row r="21" spans="1:17" s="118" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A21" s="111" t="s">
+      <c r="N20" s="113"/>
+      <c r="O20" s="104"/>
+      <c r="P20" s="104"/>
+      <c r="Q20" s="104"/>
+    </row>
+    <row r="21" spans="1:17" s="114" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A21" s="107" t="s">
         <v>223</v>
       </c>
-      <c r="B21" s="119" t="s">
+      <c r="B21" s="115" t="s">
         <v>224</v>
       </c>
-      <c r="C21" s="111" t="s">
+      <c r="C21" s="107" t="s">
         <v>114</v>
       </c>
-      <c r="D21" s="98" t="s">
+      <c r="D21" s="94" t="s">
         <v>226</v>
       </c>
-      <c r="E21" s="115" t="s">
+      <c r="E21" s="111" t="s">
         <v>237</v>
       </c>
-      <c r="F21" s="98" t="s">
+      <c r="F21" s="94" t="s">
         <v>225</v>
       </c>
-      <c r="G21" s="98" t="s">
+      <c r="G21" s="94" t="s">
         <v>227</v>
       </c>
-      <c r="H21" s="109" t="s">
+      <c r="H21" s="105" t="s">
         <v>228</v>
       </c>
-      <c r="I21" s="110" t="s">
+      <c r="I21" s="106" t="s">
         <v>72</v>
       </c>
-      <c r="J21" s="112"/>
-      <c r="K21" s="112"/>
-      <c r="L21" s="113" t="s">
+      <c r="J21" s="108"/>
+      <c r="K21" s="108"/>
+      <c r="L21" s="109" t="s">
         <v>229</v>
       </c>
-      <c r="M21" s="113" t="s">
+      <c r="M21" s="109" t="s">
         <v>63</v>
       </c>
-      <c r="N21" s="120"/>
-      <c r="O21" s="108"/>
-      <c r="P21" s="108" t="s">
+      <c r="N21" s="116"/>
+      <c r="O21" s="104"/>
+      <c r="P21" s="104" t="s">
         <v>230</v>
       </c>
-      <c r="Q21" s="108" t="s">
+      <c r="Q21" s="104" t="s">
         <v>231</v>
       </c>
     </row>
-    <row r="22" spans="1:17" s="118" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="111" t="s">
+    <row r="22" spans="1:17" s="114" customFormat="1" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A22" s="107" t="s">
         <v>295</v>
       </c>
-      <c r="B22" s="119" t="s">
+      <c r="B22" s="115" t="s">
         <v>233</v>
       </c>
-      <c r="C22" s="111" t="s">
+      <c r="C22" s="107" t="s">
         <v>114</v>
       </c>
-      <c r="D22" s="98" t="s">
+      <c r="D22" s="94" t="s">
         <v>236</v>
       </c>
-      <c r="E22" s="115" t="s">
+      <c r="E22" s="111" t="s">
         <v>234</v>
       </c>
-      <c r="F22" s="98" t="s">
+      <c r="F22" s="94" t="s">
         <v>235</v>
       </c>
-      <c r="G22" s="98" t="s">
+      <c r="G22" s="94" t="s">
         <v>227</v>
       </c>
-      <c r="H22" s="109" t="s">
+      <c r="H22" s="105" t="s">
         <v>232</v>
       </c>
-      <c r="I22" s="110" t="s">
+      <c r="I22" s="106" t="s">
         <v>72</v>
       </c>
-      <c r="J22" s="112"/>
-      <c r="K22" s="112"/>
-      <c r="L22" s="113" t="s">
+      <c r="J22" s="108"/>
+      <c r="K22" s="108"/>
+      <c r="L22" s="109" t="s">
         <v>229</v>
       </c>
-      <c r="M22" s="113" t="s">
+      <c r="M22" s="109" t="s">
         <v>63</v>
       </c>
-      <c r="N22" s="120"/>
-      <c r="O22" s="108"/>
-      <c r="P22" s="108"/>
-      <c r="Q22" s="108"/>
-    </row>
-    <row r="23" spans="1:17" s="118" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A23" s="111" t="s">
+      <c r="N22" s="116"/>
+      <c r="O22" s="104"/>
+      <c r="P22" s="104"/>
+      <c r="Q22" s="104"/>
+    </row>
+    <row r="23" spans="1:17" s="114" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A23" s="107" t="s">
         <v>296</v>
       </c>
-      <c r="B23" s="111" t="s">
+      <c r="B23" s="107" t="s">
         <v>309</v>
       </c>
-      <c r="C23" s="111" t="s">
+      <c r="C23" s="107" t="s">
         <v>114</v>
       </c>
-      <c r="D23" s="98" t="s">
+      <c r="D23" s="94" t="s">
         <v>240</v>
       </c>
-      <c r="E23" s="115" t="s">
+      <c r="E23" s="111" t="s">
         <v>238</v>
       </c>
-      <c r="F23" s="98" t="s">
+      <c r="F23" s="94" t="s">
         <v>239</v>
       </c>
-      <c r="G23" s="98"/>
-      <c r="H23" s="109" t="s">
+      <c r="G23" s="94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H23" s="105" t="s">
         <v>241</v>
       </c>
-      <c r="I23" s="110"/>
-      <c r="J23" s="112"/>
-      <c r="K23" s="112"/>
-      <c r="L23" s="113" t="s">
+      <c r="I23" s="106"/>
+      <c r="J23" s="108"/>
+      <c r="K23" s="108"/>
+      <c r="L23" s="109" t="s">
         <v>229</v>
       </c>
-      <c r="M23" s="113" t="s">
+      <c r="M23" s="109" t="s">
         <v>63</v>
       </c>
-      <c r="N23" s="120"/>
-      <c r="O23" s="108"/>
-      <c r="P23" s="108"/>
-      <c r="Q23" s="108"/>
-    </row>
-    <row r="24" spans="1:17" s="118" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A24" s="111" t="s">
+      <c r="N23" s="116"/>
+      <c r="O23" s="104"/>
+      <c r="P23" s="104"/>
+      <c r="Q23" s="104"/>
+    </row>
+    <row r="24" spans="1:17" s="114" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A24" s="107" t="s">
         <v>297</v>
       </c>
-      <c r="B24" s="111" t="s">
+      <c r="B24" s="107" t="s">
         <v>310</v>
       </c>
-      <c r="C24" s="111" t="s">
+      <c r="C24" s="107" t="s">
         <v>112</v>
       </c>
-      <c r="D24" s="98" t="s">
+      <c r="D24" s="94" t="s">
         <v>246</v>
       </c>
-      <c r="E24" s="115" t="s">
+      <c r="E24" s="111" t="s">
         <v>242</v>
       </c>
-      <c r="F24" s="98" t="s">
+      <c r="F24" s="94" t="s">
         <v>243</v>
       </c>
-      <c r="G24" s="98"/>
-      <c r="H24" s="109" t="s">
+      <c r="G24" s="94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H24" s="105" t="s">
         <v>244</v>
       </c>
-      <c r="I24" s="110"/>
-      <c r="J24" s="112"/>
-      <c r="K24" s="112"/>
-      <c r="L24" s="113" t="s">
+      <c r="I24" s="106"/>
+      <c r="J24" s="108"/>
+      <c r="K24" s="108"/>
+      <c r="L24" s="109" t="s">
         <v>229</v>
       </c>
-      <c r="M24" s="113" t="s">
+      <c r="M24" s="109" t="s">
         <v>63</v>
       </c>
-      <c r="N24" s="120"/>
-      <c r="O24" s="108" t="s">
+      <c r="N24" s="116"/>
+      <c r="O24" s="104" t="s">
         <v>245</v>
       </c>
-      <c r="P24" s="108"/>
-      <c r="Q24" s="108"/>
-    </row>
-    <row r="25" spans="1:17" s="118" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A25" s="111" t="s">
+      <c r="P24" s="104"/>
+      <c r="Q24" s="104"/>
+    </row>
+    <row r="25" spans="1:17" s="114" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A25" s="107" t="s">
         <v>298</v>
       </c>
-      <c r="B25" s="111" t="s">
+      <c r="B25" s="107" t="s">
         <v>311</v>
       </c>
-      <c r="C25" s="111" t="s">
+      <c r="C25" s="107" t="s">
         <v>114</v>
       </c>
-      <c r="D25" s="98" t="s">
+      <c r="D25" s="94" t="s">
         <v>250</v>
       </c>
-      <c r="E25" s="115" t="s">
+      <c r="E25" s="111" t="s">
         <v>321</v>
       </c>
-      <c r="F25" s="98" t="s">
+      <c r="F25" s="94" t="s">
         <v>251</v>
       </c>
-      <c r="G25" s="98"/>
-      <c r="H25" s="109" t="s">
+      <c r="G25" s="94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H25" s="105" t="s">
         <v>252</v>
       </c>
-      <c r="I25" s="110"/>
-      <c r="J25" s="112"/>
-      <c r="K25" s="112"/>
-      <c r="L25" s="113" t="s">
+      <c r="I25" s="106"/>
+      <c r="J25" s="108"/>
+      <c r="K25" s="108"/>
+      <c r="L25" s="109" t="s">
         <v>229</v>
       </c>
-      <c r="M25" s="113" t="s">
+      <c r="M25" s="109" t="s">
         <v>63</v>
       </c>
-      <c r="N25" s="120"/>
-      <c r="O25" s="108"/>
-      <c r="P25" s="108"/>
-      <c r="Q25" s="108"/>
-    </row>
-    <row r="26" spans="1:17" s="118" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A26" s="111" t="s">
+      <c r="N25" s="116"/>
+      <c r="O25" s="104"/>
+      <c r="P25" s="104"/>
+      <c r="Q25" s="104"/>
+    </row>
+    <row r="26" spans="1:17" s="114" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A26" s="107" t="s">
         <v>299</v>
       </c>
-      <c r="B26" s="111" t="s">
+      <c r="B26" s="107" t="s">
         <v>312</v>
       </c>
-      <c r="C26" s="111" t="s">
+      <c r="C26" s="107" t="s">
         <v>114</v>
       </c>
-      <c r="D26" s="98" t="s">
+      <c r="D26" s="94" t="s">
         <v>248</v>
       </c>
-      <c r="E26" s="115" t="s">
+      <c r="E26" s="111" t="s">
         <v>322</v>
       </c>
-      <c r="F26" s="98" t="s">
+      <c r="F26" s="94" t="s">
         <v>247</v>
       </c>
-      <c r="G26" s="98"/>
-      <c r="H26" s="109" t="s">
+      <c r="G26" s="94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H26" s="105" t="s">
         <v>249</v>
       </c>
-      <c r="I26" s="110"/>
-      <c r="J26" s="112"/>
-      <c r="K26" s="112"/>
-      <c r="L26" s="113" t="s">
+      <c r="I26" s="106"/>
+      <c r="J26" s="108"/>
+      <c r="K26" s="108"/>
+      <c r="L26" s="109" t="s">
         <v>229</v>
       </c>
-      <c r="M26" s="113" t="s">
+      <c r="M26" s="109" t="s">
         <v>63</v>
       </c>
-      <c r="N26" s="120"/>
-      <c r="O26" s="108"/>
-      <c r="P26" s="108"/>
-      <c r="Q26" s="108"/>
-    </row>
-    <row r="27" spans="1:17" s="118" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A27" s="111" t="s">
+      <c r="N26" s="116"/>
+      <c r="O26" s="104"/>
+      <c r="P26" s="104"/>
+      <c r="Q26" s="104"/>
+    </row>
+    <row r="27" spans="1:17" s="114" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A27" s="107" t="s">
         <v>300</v>
       </c>
-      <c r="B27" s="111" t="s">
+      <c r="B27" s="107" t="s">
         <v>313</v>
       </c>
-      <c r="C27" s="111" t="s">
+      <c r="C27" s="107" t="s">
         <v>114</v>
       </c>
-      <c r="D27" s="98" t="s">
+      <c r="D27" s="94" t="s">
         <v>255</v>
       </c>
-      <c r="E27" s="115" t="s">
+      <c r="E27" s="111" t="s">
         <v>253</v>
       </c>
-      <c r="F27" s="98" t="s">
+      <c r="F27" s="94" t="s">
         <v>254</v>
       </c>
-      <c r="G27" s="98"/>
-      <c r="H27" s="109" t="s">
+      <c r="G27" s="94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H27" s="105" t="s">
         <v>257</v>
       </c>
-      <c r="I27" s="110"/>
-      <c r="J27" s="112"/>
-      <c r="K27" s="112"/>
-      <c r="L27" s="113" t="s">
+      <c r="I27" s="106"/>
+      <c r="J27" s="108"/>
+      <c r="K27" s="108"/>
+      <c r="L27" s="109" t="s">
         <v>289</v>
       </c>
-      <c r="M27" s="113" t="s">
+      <c r="M27" s="109" t="s">
         <v>256</v>
       </c>
-      <c r="N27" s="120"/>
-      <c r="O27" s="108"/>
-      <c r="P27" s="108"/>
-      <c r="Q27" s="108"/>
-    </row>
-    <row r="28" spans="1:17" s="118" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
-      <c r="A28" s="111" t="s">
+      <c r="N27" s="116"/>
+      <c r="O27" s="104"/>
+      <c r="P27" s="104"/>
+      <c r="Q27" s="104"/>
+    </row>
+    <row r="28" spans="1:17" s="114" customFormat="1" ht="76.5" x14ac:dyDescent="0.2">
+      <c r="A28" s="107" t="s">
         <v>301</v>
       </c>
-      <c r="B28" s="111" t="s">
+      <c r="B28" s="107" t="s">
         <v>314</v>
       </c>
-      <c r="C28" s="111" t="s">
+      <c r="C28" s="107" t="s">
         <v>114</v>
       </c>
-      <c r="D28" s="98" t="s">
+      <c r="D28" s="94" t="s">
         <v>261</v>
       </c>
-      <c r="E28" s="115" t="s">
+      <c r="E28" s="111" t="s">
         <v>258</v>
       </c>
-      <c r="F28" s="98" t="s">
+      <c r="F28" s="94" t="s">
         <v>262</v>
       </c>
-      <c r="G28" s="98"/>
-      <c r="H28" s="109" t="s">
+      <c r="G28" s="94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H28" s="105" t="s">
         <v>259</v>
       </c>
-      <c r="I28" s="110"/>
-      <c r="J28" s="112"/>
-      <c r="K28" s="112"/>
-      <c r="L28" s="113" t="s">
+      <c r="I28" s="106"/>
+      <c r="J28" s="108"/>
+      <c r="K28" s="108"/>
+      <c r="L28" s="109" t="s">
         <v>289</v>
       </c>
-      <c r="M28" s="113" t="s">
+      <c r="M28" s="109" t="s">
         <v>260</v>
       </c>
-      <c r="N28" s="120"/>
-      <c r="O28" s="108" t="s">
+      <c r="N28" s="116"/>
+      <c r="O28" s="104" t="s">
         <v>263</v>
       </c>
-      <c r="P28" s="108"/>
-      <c r="Q28" s="108"/>
-    </row>
-    <row r="29" spans="1:17" s="118" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A29" s="111" t="s">
+      <c r="P28" s="104"/>
+      <c r="Q28" s="104"/>
+    </row>
+    <row r="29" spans="1:17" s="114" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A29" s="107" t="s">
         <v>302</v>
       </c>
-      <c r="B29" s="111" t="s">
+      <c r="B29" s="107" t="s">
         <v>315</v>
       </c>
-      <c r="C29" s="111" t="s">
+      <c r="C29" s="107" t="s">
         <v>113</v>
       </c>
-      <c r="D29" s="98" t="s">
+      <c r="D29" s="94" t="s">
         <v>266</v>
       </c>
-      <c r="E29" s="115" t="s">
+      <c r="E29" s="111" t="s">
         <v>264</v>
       </c>
-      <c r="F29" s="98" t="s">
+      <c r="F29" s="94" t="s">
         <v>265</v>
       </c>
-      <c r="G29" s="98"/>
-      <c r="H29" s="109" t="s">
+      <c r="G29" s="94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H29" s="105" t="s">
         <v>267</v>
       </c>
-      <c r="I29" s="110"/>
-      <c r="J29" s="112"/>
-      <c r="K29" s="112"/>
-      <c r="L29" s="113" t="s">
+      <c r="I29" s="106"/>
+      <c r="J29" s="108"/>
+      <c r="K29" s="108"/>
+      <c r="L29" s="109" t="s">
         <v>289</v>
       </c>
-      <c r="M29" s="113" t="s">
+      <c r="M29" s="109" t="s">
         <v>260</v>
       </c>
-      <c r="N29" s="120"/>
-      <c r="O29" s="108"/>
-      <c r="P29" s="108"/>
-      <c r="Q29" s="108"/>
-    </row>
-    <row r="30" spans="1:17" s="118" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A30" s="111" t="s">
+      <c r="N29" s="116"/>
+      <c r="O29" s="104"/>
+      <c r="P29" s="104"/>
+      <c r="Q29" s="104"/>
+    </row>
+    <row r="30" spans="1:17" s="114" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A30" s="107" t="s">
         <v>303</v>
       </c>
-      <c r="B30" s="111" t="s">
+      <c r="B30" s="107" t="s">
         <v>316</v>
       </c>
-      <c r="C30" s="111" t="s">
+      <c r="C30" s="107" t="s">
         <v>113</v>
       </c>
-      <c r="D30" s="98" t="s">
+      <c r="D30" s="94" t="s">
         <v>276</v>
       </c>
-      <c r="E30" s="115" t="s">
+      <c r="E30" s="111" t="s">
         <v>268</v>
       </c>
-      <c r="F30" s="98" t="s">
+      <c r="F30" s="94" t="s">
         <v>269</v>
       </c>
-      <c r="G30" s="98"/>
-      <c r="H30" s="109" t="s">
+      <c r="G30" s="94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H30" s="105" t="s">
         <v>271</v>
       </c>
-      <c r="I30" s="110"/>
-      <c r="J30" s="112"/>
-      <c r="K30" s="112"/>
-      <c r="L30" s="113" t="s">
+      <c r="I30" s="106"/>
+      <c r="J30" s="108"/>
+      <c r="K30" s="108"/>
+      <c r="L30" s="109" t="s">
         <v>39</v>
       </c>
-      <c r="M30" s="113" t="s">
+      <c r="M30" s="109" t="s">
         <v>63</v>
       </c>
-      <c r="N30" s="120"/>
-      <c r="O30" s="108"/>
-      <c r="P30" s="108"/>
-      <c r="Q30" s="108"/>
-    </row>
-    <row r="31" spans="1:17" s="118" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A31" s="111" t="s">
+      <c r="N30" s="116"/>
+      <c r="O30" s="104"/>
+      <c r="P30" s="104"/>
+      <c r="Q30" s="104"/>
+    </row>
+    <row r="31" spans="1:17" s="114" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A31" s="107" t="s">
         <v>304</v>
       </c>
-      <c r="B31" s="111" t="s">
+      <c r="B31" s="107" t="s">
         <v>317</v>
       </c>
-      <c r="C31" s="111" t="s">
+      <c r="C31" s="107" t="s">
         <v>113</v>
       </c>
-      <c r="D31" s="98" t="s">
+      <c r="D31" s="94" t="s">
         <v>277</v>
       </c>
-      <c r="E31" s="115" t="s">
+      <c r="E31" s="111" t="s">
         <v>270</v>
       </c>
-      <c r="F31" s="98" t="s">
+      <c r="F31" s="94" t="s">
         <v>269</v>
       </c>
-      <c r="G31" s="98"/>
-      <c r="H31" s="109" t="s">
+      <c r="G31" s="94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H31" s="105" t="s">
         <v>271</v>
       </c>
-      <c r="I31" s="110"/>
-      <c r="J31" s="112"/>
-      <c r="K31" s="112"/>
-      <c r="L31" s="113" t="s">
+      <c r="I31" s="106"/>
+      <c r="J31" s="108"/>
+      <c r="K31" s="108"/>
+      <c r="L31" s="109" t="s">
         <v>37</v>
       </c>
-      <c r="M31" s="113" t="s">
+      <c r="M31" s="109" t="s">
         <v>63</v>
       </c>
-      <c r="N31" s="120"/>
-      <c r="O31" s="108"/>
-      <c r="P31" s="108"/>
-      <c r="Q31" s="108"/>
-    </row>
-    <row r="32" spans="1:17" s="118" customFormat="1" ht="51" x14ac:dyDescent="0.2">
-      <c r="A32" s="111" t="s">
+      <c r="N31" s="116"/>
+      <c r="O31" s="104"/>
+      <c r="P31" s="104"/>
+      <c r="Q31" s="104"/>
+    </row>
+    <row r="32" spans="1:17" s="114" customFormat="1" ht="51" x14ac:dyDescent="0.2">
+      <c r="A32" s="107" t="s">
         <v>305</v>
       </c>
-      <c r="B32" s="111" t="s">
+      <c r="B32" s="107" t="s">
         <v>305</v>
       </c>
-      <c r="C32" s="111" t="s">
+      <c r="C32" s="107" t="s">
         <v>113</v>
       </c>
-      <c r="D32" s="98" t="s">
+      <c r="D32" s="94" t="s">
         <v>278</v>
       </c>
-      <c r="E32" s="115" t="s">
+      <c r="E32" s="111" t="s">
         <v>272</v>
       </c>
-      <c r="F32" s="98" t="s">
+      <c r="F32" s="94" t="s">
         <v>269</v>
       </c>
-      <c r="G32" s="98"/>
-      <c r="H32" s="109" t="s">
+      <c r="G32" s="94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H32" s="105" t="s">
         <v>273</v>
       </c>
-      <c r="I32" s="110"/>
-      <c r="J32" s="112"/>
-      <c r="K32" s="112"/>
-      <c r="L32" s="113" t="s">
+      <c r="I32" s="106"/>
+      <c r="J32" s="108"/>
+      <c r="K32" s="108"/>
+      <c r="L32" s="109" t="s">
         <v>289</v>
       </c>
-      <c r="M32" s="113" t="s">
+      <c r="M32" s="109" t="s">
         <v>63</v>
       </c>
-      <c r="N32" s="120"/>
-      <c r="O32" s="108" t="s">
+      <c r="N32" s="116"/>
+      <c r="O32" s="104" t="s">
         <v>274</v>
       </c>
-      <c r="P32" s="108"/>
-      <c r="Q32" s="108"/>
-    </row>
-    <row r="33" spans="1:17" s="118" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A33" s="111" t="s">
+      <c r="P32" s="104"/>
+      <c r="Q32" s="104"/>
+    </row>
+    <row r="33" spans="1:17" s="114" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A33" s="107" t="s">
         <v>306</v>
       </c>
-      <c r="B33" s="111" t="s">
+      <c r="B33" s="107" t="s">
         <v>318</v>
       </c>
-      <c r="C33" s="111" t="s">
+      <c r="C33" s="107" t="s">
         <v>113</v>
       </c>
-      <c r="D33" s="98" t="s">
+      <c r="D33" s="94" t="s">
         <v>282</v>
       </c>
-      <c r="E33" s="115" t="s">
+      <c r="E33" s="111" t="s">
         <v>279</v>
       </c>
-      <c r="F33" s="98" t="s">
+      <c r="F33" s="94" t="s">
         <v>281</v>
       </c>
-      <c r="G33" s="98"/>
-      <c r="H33" s="109" t="s">
+      <c r="G33" s="94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H33" s="105" t="s">
         <v>284</v>
       </c>
-      <c r="I33" s="110"/>
-      <c r="J33" s="112"/>
-      <c r="K33" s="112"/>
-      <c r="L33" s="113" t="s">
+      <c r="I33" s="106"/>
+      <c r="J33" s="108"/>
+      <c r="K33" s="108"/>
+      <c r="L33" s="109" t="s">
         <v>289</v>
       </c>
-      <c r="M33" s="113" t="s">
+      <c r="M33" s="109" t="s">
         <v>290</v>
       </c>
-      <c r="N33" s="120"/>
-      <c r="O33" s="108"/>
-      <c r="P33" s="108"/>
-      <c r="Q33" s="108"/>
-    </row>
-    <row r="34" spans="1:17" s="118" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A34" s="111" t="s">
+      <c r="N33" s="116"/>
+      <c r="O33" s="104"/>
+      <c r="P33" s="104"/>
+      <c r="Q33" s="104"/>
+    </row>
+    <row r="34" spans="1:17" s="114" customFormat="1" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A34" s="107" t="s">
         <v>307</v>
       </c>
-      <c r="B34" s="111" t="s">
+      <c r="B34" s="107" t="s">
         <v>319</v>
       </c>
-      <c r="C34" s="111" t="s">
+      <c r="C34" s="107" t="s">
         <v>113</v>
       </c>
-      <c r="D34" s="98" t="s">
+      <c r="D34" s="94" t="s">
         <v>283</v>
       </c>
-      <c r="E34" s="115" t="s">
+      <c r="E34" s="111" t="s">
         <v>280</v>
       </c>
-      <c r="F34" s="98" t="s">
+      <c r="F34" s="94" t="s">
         <v>281</v>
       </c>
-      <c r="G34" s="98"/>
-      <c r="H34" s="109" t="s">
+      <c r="G34" s="94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H34" s="105" t="s">
         <v>284</v>
       </c>
-      <c r="I34" s="110"/>
-      <c r="J34" s="112"/>
-      <c r="K34" s="112"/>
-      <c r="L34" s="113" t="s">
+      <c r="I34" s="106"/>
+      <c r="J34" s="108"/>
+      <c r="K34" s="108"/>
+      <c r="L34" s="109" t="s">
         <v>289</v>
       </c>
-      <c r="M34" s="113" t="s">
+      <c r="M34" s="109" t="s">
         <v>290</v>
       </c>
-      <c r="N34" s="120"/>
-      <c r="O34" s="108"/>
-      <c r="P34" s="108"/>
-      <c r="Q34" s="108"/>
-    </row>
-    <row r="35" spans="1:17" s="118" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
-      <c r="A35" s="111" t="s">
+      <c r="N34" s="116"/>
+      <c r="O34" s="104"/>
+      <c r="P34" s="104"/>
+      <c r="Q34" s="104"/>
+    </row>
+    <row r="35" spans="1:17" s="114" customFormat="1" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A35" s="107" t="s">
         <v>308</v>
       </c>
-      <c r="B35" s="111" t="s">
+      <c r="B35" s="107" t="s">
         <v>320</v>
       </c>
-      <c r="C35" s="111" t="s">
+      <c r="C35" s="107" t="s">
         <v>114</v>
       </c>
-      <c r="D35" s="98" t="s">
+      <c r="D35" s="94" t="s">
         <v>286</v>
       </c>
-      <c r="E35" s="115" t="s">
+      <c r="E35" s="111" t="s">
         <v>287</v>
       </c>
-      <c r="F35" s="98" t="s">
+      <c r="F35" s="94" t="s">
         <v>285</v>
       </c>
-      <c r="G35" s="98"/>
-      <c r="H35" s="109" t="s">
+      <c r="G35" s="94" t="s">
+        <v>227</v>
+      </c>
+      <c r="H35" s="105" t="s">
         <v>288</v>
       </c>
-      <c r="I35" s="110"/>
-      <c r="J35" s="112"/>
-      <c r="K35" s="112"/>
-      <c r="L35" s="113" t="s">
+      <c r="I35" s="106"/>
+      <c r="J35" s="108"/>
+      <c r="K35" s="108"/>
+      <c r="L35" s="109" t="s">
         <v>289</v>
       </c>
-      <c r="M35" s="113" t="s">
+      <c r="M35" s="109" t="s">
         <v>290</v>
       </c>
-      <c r="N35" s="120"/>
-      <c r="O35" s="108"/>
-      <c r="P35" s="108"/>
-      <c r="Q35" s="108"/>
+      <c r="N35" s="116"/>
+      <c r="O35" s="104"/>
+      <c r="P35" s="104"/>
+      <c r="Q35" s="104"/>
     </row>
     <row r="36" spans="1:17" x14ac:dyDescent="0.2">
       <c r="A36" s="40"/>
@@ -5060,7 +5086,7 @@
       <c r="L104" s="33"/>
       <c r="M104" s="33"/>
       <c r="N104" s="79"/>
-      <c r="O104" s="108"/>
+      <c r="O104" s="104"/>
     </row>
     <row r="105" spans="1:15" s="2" customFormat="1" ht="15" x14ac:dyDescent="0.25">
       <c r="A105" s="41"/>
@@ -5077,7 +5103,7 @@
       <c r="L105" s="33"/>
       <c r="M105" s="33"/>
       <c r="N105" s="79"/>
-      <c r="O105" s="108"/>
+      <c r="O105" s="104"/>
     </row>
     <row r="106" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A106" s="40"/>

</xml_diff>